<commit_message>
Presupuesto: valores calculados visibles (cache) conservando formulas vivas y formato
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/Solucion/PRESUPUESTO CDI TESALIA - MODULO 1 (obra gris).xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/Solucion/PRESUPUESTO CDI TESALIA - MODULO 1 (obra gris).xlsx
@@ -1827,11 +1827,11 @@
       </c>
       <c r="E5" s="16">
         <f>INSUMOS!$E$27</f>
-        <v/>
+        <v>155000.0</v>
       </c>
       <c r="F5" s="16">
         <f>D5*E5</f>
-        <v/>
+        <v>18600.0</v>
       </c>
     </row>
     <row r="6">
@@ -1855,11 +1855,11 @@
       </c>
       <c r="E6" s="16">
         <f>INSUMOS!$E$28</f>
-        <v/>
+        <v>30000.0</v>
       </c>
       <c r="F6" s="16">
         <f>D6*E6</f>
-        <v/>
+        <v>37500.0</v>
       </c>
     </row>
     <row r="7">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="E7" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F7" s="16">
         <f>D7*E7</f>
-        <v/>
+        <v>1750.3500000000001</v>
       </c>
     </row>
     <row r="8">
@@ -1912,7 +1912,7 @@
       <c r="E8" s="14" t="n"/>
       <c r="F8" s="16">
         <f>(F7)*0.05</f>
-        <v/>
+        <v>87.51750000000001</v>
       </c>
     </row>
     <row r="9">
@@ -1927,7 +1927,7 @@
       <c r="E9" s="23" t="n"/>
       <c r="F9" s="25">
         <f>SUM(F5:F8)</f>
-        <v/>
+        <v>57937.8675</v>
       </c>
     </row>
     <row r="11">
@@ -2003,11 +2003,11 @@
       </c>
       <c r="E13" s="16">
         <f>INSUMOS!$E$18</f>
-        <v/>
+        <v>95000.0</v>
       </c>
       <c r="F13" s="16">
         <f>D13*E13</f>
-        <v/>
+        <v>118750.0</v>
       </c>
     </row>
     <row r="14">
@@ -2031,11 +2031,11 @@
       </c>
       <c r="E14" s="16">
         <f>INSUMOS!$E$31</f>
-        <v/>
+        <v>62000.0</v>
       </c>
       <c r="F14" s="16">
         <f>D14*E14</f>
-        <v/>
+        <v>1550.0</v>
       </c>
     </row>
     <row r="15">
@@ -2059,11 +2059,11 @@
       </c>
       <c r="E15" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F15" s="16">
         <f>D15*E15</f>
-        <v/>
+        <v>3625.0</v>
       </c>
     </row>
     <row r="16">
@@ -2087,11 +2087,11 @@
       </c>
       <c r="E16" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F16" s="16">
         <f>D16*E16</f>
-        <v/>
+        <v>5250.0</v>
       </c>
     </row>
     <row r="17">
@@ -2116,7 +2116,7 @@
       <c r="E17" s="14" t="n"/>
       <c r="F17" s="16">
         <f>(F15+F16)*0.05</f>
-        <v/>
+        <v>443.75</v>
       </c>
     </row>
     <row r="18">
@@ -2131,7 +2131,7 @@
       <c r="E18" s="23" t="n"/>
       <c r="F18" s="25">
         <f>SUM(F13:F17)</f>
-        <v/>
+        <v>129618.75</v>
       </c>
     </row>
     <row r="20">
@@ -2207,11 +2207,11 @@
       </c>
       <c r="E22" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F22" s="16">
         <f>D22*E22</f>
-        <v/>
+        <v>34999.65</v>
       </c>
     </row>
     <row r="23">
@@ -2235,11 +2235,11 @@
       </c>
       <c r="E23" s="16">
         <f>INSUMOS!$E$28</f>
-        <v/>
+        <v>30000.0</v>
       </c>
       <c r="F23" s="16">
         <f>D23*E23</f>
-        <v/>
+        <v>37500.0</v>
       </c>
     </row>
     <row r="24">
@@ -2264,7 +2264,7 @@
       <c r="E24" s="14" t="n"/>
       <c r="F24" s="16">
         <f>(F22)*0.05</f>
-        <v/>
+        <v>1749.9825</v>
       </c>
     </row>
     <row r="25">
@@ -2279,7 +2279,7 @@
       <c r="E25" s="23" t="n"/>
       <c r="F25" s="25">
         <f>SUM(F22:F24)</f>
-        <v/>
+        <v>74249.63249999999</v>
       </c>
     </row>
     <row r="27">
@@ -2355,11 +2355,11 @@
       </c>
       <c r="E29" s="16">
         <f>INSUMOS!$E$19</f>
-        <v/>
+        <v>65000.0</v>
       </c>
       <c r="F29" s="16">
         <f>D29*E29</f>
-        <v/>
+        <v>81250.0</v>
       </c>
     </row>
     <row r="30">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="E30" s="16">
         <f>INSUMOS!$E$31</f>
-        <v/>
+        <v>62000.0</v>
       </c>
       <c r="F30" s="16">
         <f>D30*E30</f>
-        <v/>
+        <v>1550.0</v>
       </c>
     </row>
     <row r="31">
@@ -2411,11 +2411,11 @@
       </c>
       <c r="E31" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F31" s="16">
         <f>D31*E31</f>
-        <v/>
+        <v>3625.0</v>
       </c>
     </row>
     <row r="32">
@@ -2439,11 +2439,11 @@
       </c>
       <c r="E32" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F32" s="16">
         <f>D32*E32</f>
-        <v/>
+        <v>5250.0</v>
       </c>
     </row>
     <row r="33">
@@ -2468,7 +2468,7 @@
       <c r="E33" s="14" t="n"/>
       <c r="F33" s="16">
         <f>(F31+F32)*0.05</f>
-        <v/>
+        <v>443.75</v>
       </c>
     </row>
     <row r="34">
@@ -2483,7 +2483,7 @@
       <c r="E34" s="23" t="n"/>
       <c r="F34" s="25">
         <f>SUM(F29:F33)</f>
-        <v/>
+        <v>92118.75</v>
       </c>
     </row>
     <row r="36">
@@ -2559,11 +2559,11 @@
       </c>
       <c r="E38" s="16">
         <f>INSUMOS!$E$17</f>
-        <v/>
+        <v>4500.0</v>
       </c>
       <c r="F38" s="16">
         <f>D38*E38</f>
-        <v/>
+        <v>4950.0</v>
       </c>
     </row>
     <row r="39">
@@ -2587,11 +2587,11 @@
       </c>
       <c r="E39" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F39" s="16">
         <f>D39*E39</f>
-        <v/>
+        <v>874.6500000000001</v>
       </c>
     </row>
     <row r="40">
@@ -2616,7 +2616,7 @@
       <c r="E40" s="14" t="n"/>
       <c r="F40" s="16">
         <f>(F39)*0.05</f>
-        <v/>
+        <v>43.73250000000001</v>
       </c>
     </row>
     <row r="41">
@@ -2631,7 +2631,7 @@
       <c r="E41" s="23" t="n"/>
       <c r="F41" s="25">
         <f>SUM(F38:F40)</f>
-        <v/>
+        <v>5868.3825</v>
       </c>
     </row>
     <row r="43">
@@ -2707,11 +2707,11 @@
       </c>
       <c r="E45" s="16">
         <f>INSUMOS!$E$9</f>
-        <v/>
+        <v>590000.0</v>
       </c>
       <c r="F45" s="16">
         <f>D45*E45</f>
-        <v/>
+        <v>607700.0</v>
       </c>
     </row>
     <row r="46">
@@ -2735,11 +2735,11 @@
       </c>
       <c r="E46" s="16">
         <f>INSUMOS!$E$20</f>
-        <v/>
+        <v>15000.0</v>
       </c>
       <c r="F46" s="16">
         <f>D46*E46</f>
-        <v/>
+        <v>75000.0</v>
       </c>
     </row>
     <row r="47">
@@ -2763,11 +2763,11 @@
       </c>
       <c r="E47" s="16">
         <f>INSUMOS!$E$22</f>
-        <v/>
+        <v>40000.0</v>
       </c>
       <c r="F47" s="16">
         <f>D47*E47</f>
-        <v/>
+        <v>2000.0</v>
       </c>
     </row>
     <row r="48">
@@ -2791,11 +2791,11 @@
       </c>
       <c r="E48" s="16">
         <f>INSUMOS!$E$21</f>
-        <v/>
+        <v>48000.0</v>
       </c>
       <c r="F48" s="16">
         <f>D48*E48</f>
-        <v/>
+        <v>2400.0</v>
       </c>
     </row>
     <row r="49">
@@ -2819,11 +2819,11 @@
       </c>
       <c r="E49" s="16">
         <f>INSUMOS!$E$29</f>
-        <v/>
+        <v>42000.0</v>
       </c>
       <c r="F49" s="16">
         <f>D49*E49</f>
-        <v/>
+        <v>3499.86</v>
       </c>
     </row>
     <row r="50">
@@ -2847,11 +2847,11 @@
       </c>
       <c r="E50" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F50" s="16">
         <f>D50*E50</f>
-        <v/>
+        <v>18125.0</v>
       </c>
     </row>
     <row r="51">
@@ -2875,11 +2875,11 @@
       </c>
       <c r="E51" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F51" s="16">
         <f>D51*E51</f>
-        <v/>
+        <v>26250.0</v>
       </c>
     </row>
     <row r="52">
@@ -2904,7 +2904,7 @@
       <c r="E52" s="14" t="n"/>
       <c r="F52" s="16">
         <f>(F50+F51)*0.05</f>
-        <v/>
+        <v>2218.75</v>
       </c>
     </row>
     <row r="53">
@@ -2919,7 +2919,7 @@
       <c r="E53" s="23" t="n"/>
       <c r="F53" s="25">
         <f>SUM(F45:F52)</f>
-        <v/>
+        <v>737193.61</v>
       </c>
     </row>
     <row r="55">
@@ -2995,11 +2995,11 @@
       </c>
       <c r="E57" s="16">
         <f>INSUMOS!$E$10</f>
-        <v/>
+        <v>430000.0</v>
       </c>
       <c r="F57" s="16">
         <f>D57*E57</f>
-        <v/>
+        <v>21500.0</v>
       </c>
     </row>
     <row r="58">
@@ -3023,11 +3023,11 @@
       </c>
       <c r="E58" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F58" s="16">
         <f>D58*E58</f>
-        <v/>
+        <v>1812.5</v>
       </c>
     </row>
     <row r="59">
@@ -3051,11 +3051,11 @@
       </c>
       <c r="E59" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F59" s="16">
         <f>D59*E59</f>
-        <v/>
+        <v>2625.0</v>
       </c>
     </row>
     <row r="60">
@@ -3080,7 +3080,7 @@
       <c r="E60" s="14" t="n"/>
       <c r="F60" s="16">
         <f>(F58+F59)*0.05</f>
-        <v/>
+        <v>221.875</v>
       </c>
     </row>
     <row r="61">
@@ -3095,7 +3095,7 @@
       <c r="E61" s="23" t="n"/>
       <c r="F61" s="25">
         <f>SUM(F57:F60)</f>
-        <v/>
+        <v>26159.375</v>
       </c>
     </row>
     <row r="63">
@@ -3171,11 +3171,11 @@
       </c>
       <c r="E65" s="16">
         <f>INSUMOS!$E$11</f>
-        <v/>
+        <v>4800.0</v>
       </c>
       <c r="F65" s="16">
         <f>D65*E65</f>
-        <v/>
+        <v>5040.0</v>
       </c>
     </row>
     <row r="66">
@@ -3199,11 +3199,11 @@
       </c>
       <c r="E66" s="16">
         <f>INSUMOS!$E$12</f>
-        <v/>
+        <v>7000.0</v>
       </c>
       <c r="F66" s="16">
         <f>D66*E66</f>
-        <v/>
+        <v>210.0</v>
       </c>
     </row>
     <row r="67">
@@ -3227,11 +3227,11 @@
       </c>
       <c r="E67" s="16">
         <f>INSUMOS!$E$32</f>
-        <v/>
+        <v>52000.0</v>
       </c>
       <c r="F67" s="16">
         <f>D67*E67</f>
-        <v/>
+        <v>208.0</v>
       </c>
     </row>
     <row r="68">
@@ -3255,11 +3255,11 @@
       </c>
       <c r="E68" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F68" s="16">
         <f>D68*E68</f>
-        <v/>
+        <v>580.0</v>
       </c>
     </row>
     <row r="69">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="E69" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F69" s="16">
         <f>D69*E69</f>
-        <v/>
+        <v>840.0</v>
       </c>
     </row>
     <row r="70">
@@ -3312,7 +3312,7 @@
       <c r="E70" s="14" t="n"/>
       <c r="F70" s="16">
         <f>(F68+F69)*0.05</f>
-        <v/>
+        <v>71.0</v>
       </c>
     </row>
     <row r="71">
@@ -3327,7 +3327,7 @@
       <c r="E71" s="23" t="n"/>
       <c r="F71" s="25">
         <f>SUM(F65:F70)</f>
-        <v/>
+        <v>6949.0</v>
       </c>
     </row>
     <row r="73">
@@ -3403,11 +3403,11 @@
       </c>
       <c r="E75" s="16">
         <f>INSUMOS!$E$9</f>
-        <v/>
+        <v>590000.0</v>
       </c>
       <c r="F75" s="16">
         <f>D75*E75</f>
-        <v/>
+        <v>607700.0</v>
       </c>
     </row>
     <row r="76">
@@ -3431,11 +3431,11 @@
       </c>
       <c r="E76" s="16">
         <f>INSUMOS!$E$20</f>
-        <v/>
+        <v>15000.0</v>
       </c>
       <c r="F76" s="16">
         <f>D76*E76</f>
-        <v/>
+        <v>120000.0</v>
       </c>
     </row>
     <row r="77">
@@ -3459,11 +3459,11 @@
       </c>
       <c r="E77" s="16">
         <f>INSUMOS!$E$22</f>
-        <v/>
+        <v>40000.0</v>
       </c>
       <c r="F77" s="16">
         <f>D77*E77</f>
-        <v/>
+        <v>4000.0</v>
       </c>
     </row>
     <row r="78">
@@ -3487,11 +3487,11 @@
       </c>
       <c r="E78" s="16">
         <f>INSUMOS!$E$21</f>
-        <v/>
+        <v>48000.0</v>
       </c>
       <c r="F78" s="16">
         <f>D78*E78</f>
-        <v/>
+        <v>4800.0</v>
       </c>
     </row>
     <row r="79">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="E79" s="16">
         <f>INSUMOS!$E$29</f>
-        <v/>
+        <v>42000.0</v>
       </c>
       <c r="F79" s="16">
         <f>D79*E79</f>
-        <v/>
+        <v>4200.0</v>
       </c>
     </row>
     <row r="80">
@@ -3543,11 +3543,11 @@
       </c>
       <c r="E80" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F80" s="16">
         <f>D80*E80</f>
-        <v/>
+        <v>24167.15</v>
       </c>
     </row>
     <row r="81">
@@ -3571,11 +3571,11 @@
       </c>
       <c r="E81" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F81" s="16">
         <f>D81*E81</f>
-        <v/>
+        <v>52500.0</v>
       </c>
     </row>
     <row r="82">
@@ -3600,7 +3600,7 @@
       <c r="E82" s="14" t="n"/>
       <c r="F82" s="16">
         <f>(F80+F81)*0.05</f>
-        <v/>
+        <v>3833.3575</v>
       </c>
     </row>
     <row r="83">
@@ -3615,7 +3615,7 @@
       <c r="E83" s="23" t="n"/>
       <c r="F83" s="25">
         <f>SUM(F75:F82)</f>
-        <v/>
+        <v>821200.5075000001</v>
       </c>
     </row>
     <row r="85">
@@ -3691,11 +3691,11 @@
       </c>
       <c r="E87" s="16">
         <f>INSUMOS!$E$9</f>
-        <v/>
+        <v>590000.0</v>
       </c>
       <c r="F87" s="16">
         <f>D87*E87</f>
-        <v/>
+        <v>607700.0</v>
       </c>
     </row>
     <row r="88">
@@ -3719,11 +3719,11 @@
       </c>
       <c r="E88" s="16">
         <f>INSUMOS!$E$20</f>
-        <v/>
+        <v>15000.0</v>
       </c>
       <c r="F88" s="16">
         <f>D88*E88</f>
-        <v/>
+        <v>90000.0</v>
       </c>
     </row>
     <row r="89">
@@ -3747,11 +3747,11 @@
       </c>
       <c r="E89" s="16">
         <f>INSUMOS!$E$22</f>
-        <v/>
+        <v>40000.0</v>
       </c>
       <c r="F89" s="16">
         <f>D89*E89</f>
-        <v/>
+        <v>2400.0</v>
       </c>
     </row>
     <row r="90">
@@ -3775,11 +3775,11 @@
       </c>
       <c r="E90" s="16">
         <f>INSUMOS!$E$29</f>
-        <v/>
+        <v>42000.0</v>
       </c>
       <c r="F90" s="16">
         <f>D90*E90</f>
-        <v/>
+        <v>3499.86</v>
       </c>
     </row>
     <row r="91">
@@ -3803,11 +3803,11 @@
       </c>
       <c r="E91" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F91" s="16">
         <f>D91*E91</f>
-        <v/>
+        <v>18125.0</v>
       </c>
     </row>
     <row r="92">
@@ -3831,11 +3831,11 @@
       </c>
       <c r="E92" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F92" s="16">
         <f>D92*E92</f>
-        <v/>
+        <v>26250.0</v>
       </c>
     </row>
     <row r="93">
@@ -3860,7 +3860,7 @@
       <c r="E93" s="14" t="n"/>
       <c r="F93" s="16">
         <f>(F91+F92)*0.05</f>
-        <v/>
+        <v>2218.75</v>
       </c>
     </row>
     <row r="94">
@@ -3875,7 +3875,7 @@
       <c r="E94" s="23" t="n"/>
       <c r="F94" s="25">
         <f>SUM(F87:F93)</f>
-        <v/>
+        <v>750193.61</v>
       </c>
     </row>
     <row r="96">
@@ -3951,11 +3951,11 @@
       </c>
       <c r="E98" s="16">
         <f>INSUMOS!$E$9</f>
-        <v/>
+        <v>590000.0</v>
       </c>
       <c r="F98" s="16">
         <f>D98*E98</f>
-        <v/>
+        <v>607700.0</v>
       </c>
     </row>
     <row r="99">
@@ -3979,11 +3979,11 @@
       </c>
       <c r="E99" s="16">
         <f>INSUMOS!$E$20</f>
-        <v/>
+        <v>15000.0</v>
       </c>
       <c r="F99" s="16">
         <f>D99*E99</f>
-        <v/>
+        <v>15000.0</v>
       </c>
     </row>
     <row r="100">
@@ -4007,11 +4007,11 @@
       </c>
       <c r="E100" s="16">
         <f>INSUMOS!$E$29</f>
-        <v/>
+        <v>42000.0</v>
       </c>
       <c r="F100" s="16">
         <f>D100*E100</f>
-        <v/>
+        <v>2800.14</v>
       </c>
     </row>
     <row r="101">
@@ -4035,11 +4035,11 @@
       </c>
       <c r="E101" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F101" s="16">
         <f>D101*E101</f>
-        <v/>
+        <v>12082.85</v>
       </c>
     </row>
     <row r="102">
@@ -4063,11 +4063,11 @@
       </c>
       <c r="E102" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F102" s="16">
         <f>D102*E102</f>
-        <v/>
+        <v>26250.0</v>
       </c>
     </row>
     <row r="103">
@@ -4092,7 +4092,7 @@
       <c r="E103" s="14" t="n"/>
       <c r="F103" s="16">
         <f>(F101+F102)*0.05</f>
-        <v/>
+        <v>1916.6425</v>
       </c>
     </row>
     <row r="104">
@@ -4107,7 +4107,7 @@
       <c r="E104" s="23" t="n"/>
       <c r="F104" s="25">
         <f>SUM(F98:F103)</f>
-        <v/>
+        <v>665749.6325</v>
       </c>
     </row>
     <row r="106">
@@ -4183,11 +4183,11 @@
       </c>
       <c r="E108" s="16">
         <f>INSUMOS!$E$9</f>
-        <v/>
+        <v>590000.0</v>
       </c>
       <c r="F108" s="16">
         <f>D108*E108</f>
-        <v/>
+        <v>50150.0</v>
       </c>
     </row>
     <row r="109">
@@ -4211,11 +4211,11 @@
       </c>
       <c r="E109" s="16">
         <f>INSUMOS!$E$20</f>
-        <v/>
+        <v>15000.0</v>
       </c>
       <c r="F109" s="16">
         <f>D109*E109</f>
-        <v/>
+        <v>16500.0</v>
       </c>
     </row>
     <row r="110">
@@ -4239,11 +4239,11 @@
       </c>
       <c r="E110" s="16">
         <f>INSUMOS!$E$24</f>
-        <v/>
+        <v>19000.0</v>
       </c>
       <c r="F110" s="16">
         <f>D110*E110</f>
-        <v/>
+        <v>19000.0</v>
       </c>
     </row>
     <row r="111">
@@ -4267,11 +4267,11 @@
       </c>
       <c r="E111" s="16">
         <f>INSUMOS!$E$29</f>
-        <v/>
+        <v>42000.0</v>
       </c>
       <c r="F111" s="16">
         <f>D111*E111</f>
-        <v/>
+        <v>700.14</v>
       </c>
     </row>
     <row r="112">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="E112" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F112" s="16">
         <f>D112*E112</f>
-        <v/>
+        <v>12082.85</v>
       </c>
     </row>
     <row r="113">
@@ -4323,11 +4323,11 @@
       </c>
       <c r="E113" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F113" s="16">
         <f>D113*E113</f>
-        <v/>
+        <v>26250.0</v>
       </c>
     </row>
     <row r="114">
@@ -4352,7 +4352,7 @@
       <c r="E114" s="14" t="n"/>
       <c r="F114" s="16">
         <f>(F112+F113)*0.05</f>
-        <v/>
+        <v>1916.6425</v>
       </c>
     </row>
     <row r="115">
@@ -4367,7 +4367,7 @@
       <c r="E115" s="23" t="n"/>
       <c r="F115" s="25">
         <f>SUM(F108:F114)</f>
-        <v/>
+        <v>126599.6325</v>
       </c>
     </row>
     <row r="117">
@@ -4443,11 +4443,11 @@
       </c>
       <c r="E119" s="16">
         <f>INSUMOS!$E$13</f>
-        <v/>
+        <v>6500.0</v>
       </c>
       <c r="F119" s="16">
         <f>D119*E119</f>
-        <v/>
+        <v>6825.0</v>
       </c>
     </row>
     <row r="120">
@@ -4471,11 +4471,11 @@
       </c>
       <c r="E120" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F120" s="16">
         <f>D120*E120</f>
-        <v/>
+        <v>362.5</v>
       </c>
     </row>
     <row r="121">
@@ -4499,11 +4499,11 @@
       </c>
       <c r="E121" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F121" s="16">
         <f>D121*E121</f>
-        <v/>
+        <v>262.5</v>
       </c>
     </row>
     <row r="122">
@@ -4528,7 +4528,7 @@
       <c r="E122" s="14" t="n"/>
       <c r="F122" s="16">
         <f>(F120+F121)*0.05</f>
-        <v/>
+        <v>31.25</v>
       </c>
     </row>
     <row r="123">
@@ -4543,7 +4543,7 @@
       <c r="E123" s="23" t="n"/>
       <c r="F123" s="25">
         <f>SUM(F119:F122)</f>
-        <v/>
+        <v>7481.25</v>
       </c>
     </row>
     <row r="125">
@@ -4619,11 +4619,11 @@
       </c>
       <c r="E127" s="16">
         <f>INSUMOS!$E$11</f>
-        <v/>
+        <v>4800.0</v>
       </c>
       <c r="F127" s="16">
         <f>D127*E127</f>
-        <v/>
+        <v>5040.0</v>
       </c>
     </row>
     <row r="128">
@@ -4647,11 +4647,11 @@
       </c>
       <c r="E128" s="16">
         <f>INSUMOS!$E$12</f>
-        <v/>
+        <v>7000.0</v>
       </c>
       <c r="F128" s="16">
         <f>D128*E128</f>
-        <v/>
+        <v>210.0</v>
       </c>
     </row>
     <row r="129">
@@ -4675,11 +4675,11 @@
       </c>
       <c r="E129" s="16">
         <f>INSUMOS!$E$32</f>
-        <v/>
+        <v>52000.0</v>
       </c>
       <c r="F129" s="16">
         <f>D129*E129</f>
-        <v/>
+        <v>208.0</v>
       </c>
     </row>
     <row r="130">
@@ -4703,11 +4703,11 @@
       </c>
       <c r="E130" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F130" s="16">
         <f>D130*E130</f>
-        <v/>
+        <v>580.0</v>
       </c>
     </row>
     <row r="131">
@@ -4731,11 +4731,11 @@
       </c>
       <c r="E131" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F131" s="16">
         <f>D131*E131</f>
-        <v/>
+        <v>840.0</v>
       </c>
     </row>
     <row r="132">
@@ -4760,7 +4760,7 @@
       <c r="E132" s="14" t="n"/>
       <c r="F132" s="16">
         <f>(F130+F131)*0.05</f>
-        <v/>
+        <v>71.0</v>
       </c>
     </row>
     <row r="133">
@@ -4775,7 +4775,7 @@
       <c r="E133" s="23" t="n"/>
       <c r="F133" s="25">
         <f>SUM(F127:F132)</f>
-        <v/>
+        <v>6949.0</v>
       </c>
     </row>
     <row r="135">
@@ -4851,11 +4851,11 @@
       </c>
       <c r="E137" s="16">
         <f>INSUMOS!$E$11</f>
-        <v/>
+        <v>4800.0</v>
       </c>
       <c r="F137" s="16">
         <f>D137*E137</f>
-        <v/>
+        <v>5040.0</v>
       </c>
     </row>
     <row r="138">
@@ -4879,11 +4879,11 @@
       </c>
       <c r="E138" s="16">
         <f>INSUMOS!$E$12</f>
-        <v/>
+        <v>7000.0</v>
       </c>
       <c r="F138" s="16">
         <f>D138*E138</f>
-        <v/>
+        <v>210.0</v>
       </c>
     </row>
     <row r="139">
@@ -4907,11 +4907,11 @@
       </c>
       <c r="E139" s="16">
         <f>INSUMOS!$E$32</f>
-        <v/>
+        <v>52000.0</v>
       </c>
       <c r="F139" s="16">
         <f>D139*E139</f>
-        <v/>
+        <v>208.0</v>
       </c>
     </row>
     <row r="140">
@@ -4935,11 +4935,11 @@
       </c>
       <c r="E140" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F140" s="16">
         <f>D140*E140</f>
-        <v/>
+        <v>580.0</v>
       </c>
     </row>
     <row r="141">
@@ -4963,11 +4963,11 @@
       </c>
       <c r="E141" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F141" s="16">
         <f>D141*E141</f>
-        <v/>
+        <v>840.0</v>
       </c>
     </row>
     <row r="142">
@@ -4992,7 +4992,7 @@
       <c r="E142" s="14" t="n"/>
       <c r="F142" s="16">
         <f>(F140+F141)*0.05</f>
-        <v/>
+        <v>71.0</v>
       </c>
     </row>
     <row r="143">
@@ -5007,7 +5007,7 @@
       <c r="E143" s="23" t="n"/>
       <c r="F143" s="25">
         <f>SUM(F137:F142)</f>
-        <v/>
+        <v>6949.0</v>
       </c>
     </row>
     <row r="145">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="E147" s="16">
         <f>INSUMOS!$E$13</f>
-        <v/>
+        <v>6500.0</v>
       </c>
       <c r="F147" s="16">
         <f>D147*E147</f>
-        <v/>
+        <v>6825.0</v>
       </c>
     </row>
     <row r="148">
@@ -5111,11 +5111,11 @@
       </c>
       <c r="E148" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F148" s="16">
         <f>D148*E148</f>
-        <v/>
+        <v>362.5</v>
       </c>
     </row>
     <row r="149">
@@ -5139,11 +5139,11 @@
       </c>
       <c r="E149" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F149" s="16">
         <f>D149*E149</f>
-        <v/>
+        <v>262.5</v>
       </c>
     </row>
     <row r="150">
@@ -5168,7 +5168,7 @@
       <c r="E150" s="14" t="n"/>
       <c r="F150" s="16">
         <f>(F148+F149)*0.05</f>
-        <v/>
+        <v>31.25</v>
       </c>
     </row>
     <row r="151">
@@ -5183,7 +5183,7 @@
       <c r="E151" s="23" t="n"/>
       <c r="F151" s="25">
         <f>SUM(F147:F150)</f>
-        <v/>
+        <v>7481.25</v>
       </c>
     </row>
     <row r="153">
@@ -5259,11 +5259,11 @@
       </c>
       <c r="E155" s="16">
         <f>INSUMOS!$E$14</f>
-        <v/>
+        <v>2700.0</v>
       </c>
       <c r="F155" s="16">
         <f>D155*E155</f>
-        <v/>
+        <v>33750.0</v>
       </c>
     </row>
     <row r="156">
@@ -5287,11 +5287,11 @@
       </c>
       <c r="E156" s="16">
         <f>INSUMOS!$E$4</f>
-        <v/>
+        <v>34000.0</v>
       </c>
       <c r="F156" s="16">
         <f>D156*E156</f>
-        <v/>
+        <v>4080.0</v>
       </c>
     </row>
     <row r="157">
@@ -5315,11 +5315,11 @@
       </c>
       <c r="E157" s="16">
         <f>INSUMOS!$E$5</f>
-        <v/>
+        <v>82000.0</v>
       </c>
       <c r="F157" s="16">
         <f>D157*E157</f>
-        <v/>
+        <v>1640.0</v>
       </c>
     </row>
     <row r="158">
@@ -5343,11 +5343,11 @@
       </c>
       <c r="E158" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F158" s="16">
         <f>D158*E158</f>
-        <v/>
+        <v>12082.85</v>
       </c>
     </row>
     <row r="159">
@@ -5371,11 +5371,11 @@
       </c>
       <c r="E159" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F159" s="16">
         <f>D159*E159</f>
-        <v/>
+        <v>8749.65</v>
       </c>
     </row>
     <row r="160">
@@ -5400,7 +5400,7 @@
       <c r="E160" s="14" t="n"/>
       <c r="F160" s="16">
         <f>(F158+F159)*0.05</f>
-        <v/>
+        <v>1041.625</v>
       </c>
     </row>
     <row r="161">
@@ -5415,7 +5415,7 @@
       <c r="E161" s="23" t="n"/>
       <c r="F161" s="25">
         <f>SUM(F155:F160)</f>
-        <v/>
+        <v>61344.125</v>
       </c>
     </row>
     <row r="163">
@@ -5491,11 +5491,11 @@
       </c>
       <c r="E165" s="16">
         <f>INSUMOS!$E$15</f>
-        <v/>
+        <v>3100.0</v>
       </c>
       <c r="F165" s="16">
         <f>D165*E165</f>
-        <v/>
+        <v>15500.0</v>
       </c>
     </row>
     <row r="166">
@@ -5519,11 +5519,11 @@
       </c>
       <c r="E166" s="16">
         <f>INSUMOS!$E$4</f>
-        <v/>
+        <v>34000.0</v>
       </c>
       <c r="F166" s="16">
         <f>D166*E166</f>
-        <v/>
+        <v>3400.0</v>
       </c>
     </row>
     <row r="167">
@@ -5547,11 +5547,11 @@
       </c>
       <c r="E167" s="16">
         <f>INSUMOS!$E$5</f>
-        <v/>
+        <v>82000.0</v>
       </c>
       <c r="F167" s="16">
         <f>D167*E167</f>
-        <v/>
+        <v>1230.0</v>
       </c>
     </row>
     <row r="168">
@@ -5575,11 +5575,11 @@
       </c>
       <c r="E168" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F168" s="16">
         <f>D168*E168</f>
-        <v/>
+        <v>7250.0</v>
       </c>
     </row>
     <row r="169">
@@ -5603,11 +5603,11 @@
       </c>
       <c r="E169" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F169" s="16">
         <f>D169*E169</f>
-        <v/>
+        <v>5250.0</v>
       </c>
     </row>
     <row r="170">
@@ -5632,7 +5632,7 @@
       <c r="E170" s="14" t="n"/>
       <c r="F170" s="16">
         <f>(F168+F169)*0.05</f>
-        <v/>
+        <v>625.0</v>
       </c>
     </row>
     <row r="171">
@@ -5647,7 +5647,7 @@
       <c r="E171" s="23" t="n"/>
       <c r="F171" s="25">
         <f>SUM(F165:F170)</f>
-        <v/>
+        <v>33255.0</v>
       </c>
     </row>
     <row r="173">
@@ -5723,11 +5723,11 @@
       </c>
       <c r="E175" s="16">
         <f>INSUMOS!$E$4</f>
-        <v/>
+        <v>34000.0</v>
       </c>
       <c r="F175" s="16">
         <f>D175*E175</f>
-        <v/>
+        <v>2720.0</v>
       </c>
     </row>
     <row r="176">
@@ -5751,11 +5751,11 @@
       </c>
       <c r="E176" s="16">
         <f>INSUMOS!$E$5</f>
-        <v/>
+        <v>82000.0</v>
       </c>
       <c r="F176" s="16">
         <f>D176*E176</f>
-        <v/>
+        <v>1640.0</v>
       </c>
     </row>
     <row r="177">
@@ -5779,11 +5779,11 @@
       </c>
       <c r="E177" s="16">
         <f>INSUMOS!$E$21</f>
-        <v/>
+        <v>48000.0</v>
       </c>
       <c r="F177" s="16">
         <f>D177*E177</f>
-        <v/>
+        <v>960.0</v>
       </c>
     </row>
     <row r="178">
@@ -5807,11 +5807,11 @@
       </c>
       <c r="E178" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F178" s="16">
         <f>D178*E178</f>
-        <v/>
+        <v>10357.349999999999</v>
       </c>
     </row>
     <row r="179">
@@ -5835,11 +5835,11 @@
       </c>
       <c r="E179" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F179" s="16">
         <f>D179*E179</f>
-        <v/>
+        <v>7500.15</v>
       </c>
     </row>
     <row r="180">
@@ -5864,7 +5864,7 @@
       <c r="E180" s="14" t="n"/>
       <c r="F180" s="16">
         <f>(F178+F179)*0.05</f>
-        <v/>
+        <v>892.875</v>
       </c>
     </row>
     <row r="181">
@@ -5879,7 +5879,7 @@
       <c r="E181" s="23" t="n"/>
       <c r="F181" s="25">
         <f>SUM(F175:F180)</f>
-        <v/>
+        <v>24070.375</v>
       </c>
     </row>
     <row r="183">
@@ -5955,11 +5955,11 @@
       </c>
       <c r="E185" s="16">
         <f>INSUMOS!$E$11</f>
-        <v/>
+        <v>4800.0</v>
       </c>
       <c r="F185" s="16">
         <f>D185*E185</f>
-        <v/>
+        <v>5040.0</v>
       </c>
     </row>
     <row r="186">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="E186" s="16">
         <f>INSUMOS!$E$12</f>
-        <v/>
+        <v>7000.0</v>
       </c>
       <c r="F186" s="16">
         <f>D186*E186</f>
-        <v/>
+        <v>210.0</v>
       </c>
     </row>
     <row r="187">
@@ -6011,11 +6011,11 @@
       </c>
       <c r="E187" s="16">
         <f>INSUMOS!$E$32</f>
-        <v/>
+        <v>52000.0</v>
       </c>
       <c r="F187" s="16">
         <f>D187*E187</f>
-        <v/>
+        <v>208.0</v>
       </c>
     </row>
     <row r="188">
@@ -6039,11 +6039,11 @@
       </c>
       <c r="E188" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F188" s="16">
         <f>D188*E188</f>
-        <v/>
+        <v>580.0</v>
       </c>
     </row>
     <row r="189">
@@ -6067,11 +6067,11 @@
       </c>
       <c r="E189" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F189" s="16">
         <f>D189*E189</f>
-        <v/>
+        <v>840.0</v>
       </c>
     </row>
     <row r="190">
@@ -6096,7 +6096,7 @@
       <c r="E190" s="14" t="n"/>
       <c r="F190" s="16">
         <f>(F188+F189)*0.05</f>
-        <v/>
+        <v>71.0</v>
       </c>
     </row>
     <row r="191">
@@ -6111,7 +6111,7 @@
       <c r="E191" s="23" t="n"/>
       <c r="F191" s="25">
         <f>SUM(F185:F190)</f>
-        <v/>
+        <v>6949.0</v>
       </c>
     </row>
     <row r="193">
@@ -6187,11 +6187,11 @@
       </c>
       <c r="E195" s="16">
         <f>INSUMOS!$E$16</f>
-        <v/>
+        <v>1350.0</v>
       </c>
       <c r="F195" s="16">
         <f>D195*E195</f>
-        <v/>
+        <v>67500.0</v>
       </c>
     </row>
     <row r="196">
@@ -6215,11 +6215,11 @@
       </c>
       <c r="E196" s="16">
         <f>INSUMOS!$E$23</f>
-        <v/>
+        <v>74000.0</v>
       </c>
       <c r="F196" s="16">
         <f>D196*E196</f>
-        <v/>
+        <v>3700.0</v>
       </c>
     </row>
     <row r="197">
@@ -6243,11 +6243,11 @@
       </c>
       <c r="E197" s="16">
         <f>INSUMOS!$E$5</f>
-        <v/>
+        <v>82000.0</v>
       </c>
       <c r="F197" s="16">
         <f>D197*E197</f>
-        <v/>
+        <v>820.0</v>
       </c>
     </row>
     <row r="198">
@@ -6271,11 +6271,11 @@
       </c>
       <c r="E198" s="16">
         <f>INSUMOS!$E$31</f>
-        <v/>
+        <v>62000.0</v>
       </c>
       <c r="F198" s="16">
         <f>D198*E198</f>
-        <v/>
+        <v>775.0</v>
       </c>
     </row>
     <row r="199">
@@ -6299,11 +6299,11 @@
       </c>
       <c r="E199" s="16">
         <f>INSUMOS!$E$25</f>
-        <v/>
+        <v>145000.0</v>
       </c>
       <c r="F199" s="16">
         <f>D199*E199</f>
-        <v/>
+        <v>9667.15</v>
       </c>
     </row>
     <row r="200">
@@ -6327,11 +6327,11 @@
       </c>
       <c r="E200" s="16">
         <f>INSUMOS!$E$26</f>
-        <v/>
+        <v>105000.0</v>
       </c>
       <c r="F200" s="16">
         <f>D200*E200</f>
-        <v/>
+        <v>13999.65</v>
       </c>
     </row>
     <row r="201">
@@ -6356,7 +6356,7 @@
       <c r="E201" s="14" t="n"/>
       <c r="F201" s="16">
         <f>(F199+F200)*0.05</f>
-        <v/>
+        <v>1183.34</v>
       </c>
     </row>
     <row r="202">
@@ -6371,7 +6371,7 @@
       <c r="E202" s="23" t="n"/>
       <c r="F202" s="25">
         <f>SUM(F195:F201)</f>
-        <v/>
+        <v>97645.13999999998</v>
       </c>
     </row>
   </sheetData>
@@ -6491,11 +6491,11 @@
       </c>
       <c r="E5" s="16">
         <f>APU!$F$9</f>
-        <v/>
+        <v>57937.8675</v>
       </c>
       <c r="F5" s="16">
         <f>D5*E5</f>
-        <v/>
+        <v>6889391.824425</v>
       </c>
     </row>
     <row r="6">
@@ -6519,11 +6519,11 @@
       </c>
       <c r="E6" s="16">
         <f>APU!$F$18</f>
-        <v/>
+        <v>129618.75</v>
       </c>
       <c r="F6" s="16">
         <f>D6*E6</f>
-        <v/>
+        <v>4203536.0625</v>
       </c>
     </row>
     <row r="7">
@@ -6547,11 +6547,11 @@
       </c>
       <c r="E7" s="16">
         <f>APU!$F$25</f>
-        <v/>
+        <v>74249.63249999999</v>
       </c>
       <c r="F7" s="16">
         <f>D7*E7</f>
-        <v/>
+        <v>904360.5238499999</v>
       </c>
     </row>
     <row r="8">
@@ -6575,11 +6575,11 @@
       </c>
       <c r="E8" s="16">
         <f>APU!$F$34</f>
-        <v/>
+        <v>92118.75</v>
       </c>
       <c r="F8" s="16">
         <f>D8*E8</f>
-        <v/>
+        <v>3983214.75</v>
       </c>
     </row>
     <row r="9">
@@ -6603,11 +6603,11 @@
       </c>
       <c r="E9" s="16">
         <f>APU!$F$41</f>
-        <v/>
+        <v>5868.3825</v>
       </c>
       <c r="F9" s="16">
         <f>D9*E9</f>
-        <v/>
+        <v>1268744.2965</v>
       </c>
     </row>
     <row r="10">
@@ -6647,11 +6647,11 @@
       </c>
       <c r="E11" s="16">
         <f>APU!$F$53</f>
-        <v/>
+        <v>737193.61</v>
       </c>
       <c r="F11" s="16">
         <f>D11*E11</f>
-        <v/>
+        <v>10099552.456999999</v>
       </c>
     </row>
     <row r="12">
@@ -6675,11 +6675,11 @@
       </c>
       <c r="E12" s="16">
         <f>APU!$F$61</f>
-        <v/>
+        <v>26159.375</v>
       </c>
       <c r="F12" s="16">
         <f>D12*E12</f>
-        <v/>
+        <v>995364.2187499999</v>
       </c>
     </row>
     <row r="13">
@@ -6719,11 +6719,11 @@
       </c>
       <c r="E14" s="16">
         <f>APU!$F$71</f>
-        <v/>
+        <v>6949.0</v>
       </c>
       <c r="F14" s="16">
         <f>D14*E14</f>
-        <v/>
+        <v>9051767.399999999</v>
       </c>
     </row>
     <row r="15">
@@ -6779,11 +6779,11 @@
       </c>
       <c r="E17" s="16">
         <f>APU!$F$83</f>
-        <v/>
+        <v>821200.5075000001</v>
       </c>
       <c r="F17" s="16">
         <f>D17*E17</f>
-        <v/>
+        <v>6438211.978800001</v>
       </c>
     </row>
     <row r="18">
@@ -6823,11 +6823,11 @@
       </c>
       <c r="E19" s="16">
         <f>APU!$F$94</f>
-        <v/>
+        <v>750193.61</v>
       </c>
       <c r="F19" s="16">
         <f>D19*E19</f>
-        <v/>
+        <v>11417946.7442</v>
       </c>
     </row>
     <row r="20">
@@ -6867,11 +6867,11 @@
       </c>
       <c r="E21" s="16">
         <f>APU!$F$104</f>
-        <v/>
+        <v>665749.6325</v>
       </c>
       <c r="F21" s="16">
         <f>D21*E21</f>
-        <v/>
+        <v>14393507.05465</v>
       </c>
     </row>
     <row r="22">
@@ -6895,11 +6895,11 @@
       </c>
       <c r="E22" s="16">
         <f>APU!$F$115</f>
-        <v/>
+        <v>126599.6325</v>
       </c>
       <c r="F22" s="16">
         <f>D22*E22</f>
-        <v/>
+        <v>17116270.314</v>
       </c>
     </row>
     <row r="23">
@@ -6939,11 +6939,11 @@
       </c>
       <c r="E24" s="16">
         <f>APU!$F$123</f>
-        <v/>
+        <v>7481.25</v>
       </c>
       <c r="F24" s="16">
         <f>D24*E24</f>
-        <v/>
+        <v>9370265.625</v>
       </c>
     </row>
     <row r="25">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="E26" s="16">
         <f>APU!$F$133</f>
-        <v/>
+        <v>6949.0</v>
       </c>
       <c r="F26" s="16">
         <f>D26*E26</f>
-        <v/>
+        <v>5502218.199999999</v>
       </c>
     </row>
     <row r="27">
@@ -7027,11 +7027,11 @@
       </c>
       <c r="E28" s="16">
         <f>APU!$F$143</f>
-        <v/>
+        <v>6949.0</v>
       </c>
       <c r="F28" s="16">
         <f>D28*E28</f>
-        <v/>
+        <v>12214257.3</v>
       </c>
     </row>
     <row r="29">
@@ -7071,11 +7071,11 @@
       </c>
       <c r="E30" s="16">
         <f>APU!$F$151</f>
-        <v/>
+        <v>7481.25</v>
       </c>
       <c r="F30" s="16">
         <f>D30*E30</f>
-        <v/>
+        <v>5860063.125</v>
       </c>
     </row>
     <row r="31">
@@ -7131,11 +7131,11 @@
       </c>
       <c r="E33" s="16">
         <f>APU!$F$161</f>
-        <v/>
+        <v>61344.125</v>
       </c>
       <c r="F33" s="16">
         <f>D33*E33</f>
-        <v/>
+        <v>24706346.34375</v>
       </c>
     </row>
     <row r="34">
@@ -7159,11 +7159,11 @@
       </c>
       <c r="E34" s="16">
         <f>APU!$F$171</f>
-        <v/>
+        <v>33255.0</v>
       </c>
       <c r="F34" s="16">
         <f>D34*E34</f>
-        <v/>
+        <v>5593491.0</v>
       </c>
     </row>
     <row r="35">
@@ -7187,11 +7187,11 @@
       </c>
       <c r="E35" s="16">
         <f>APU!$F$181</f>
-        <v/>
+        <v>24070.375</v>
       </c>
       <c r="F35" s="16">
         <f>D35*E35</f>
-        <v/>
+        <v>6301383.47125</v>
       </c>
     </row>
     <row r="36">
@@ -7231,11 +7231,11 @@
       </c>
       <c r="E37" s="16">
         <f>APU!$F$191</f>
-        <v/>
+        <v>6949.0</v>
       </c>
       <c r="F37" s="16">
         <f>D37*E37</f>
-        <v/>
+        <v>3683664.9000000004</v>
       </c>
     </row>
     <row r="38">
@@ -7291,11 +7291,11 @@
       </c>
       <c r="E40" s="16">
         <f>APU!$F$202</f>
-        <v/>
+        <v>97645.13999999998</v>
       </c>
       <c r="F40" s="16">
         <f>D40*E40</f>
-        <v/>
+        <v>11258484.641999997</v>
       </c>
     </row>
     <row r="41">
@@ -7310,7 +7310,7 @@
       <c r="E41" s="31" t="n"/>
       <c r="F41" s="33">
         <f>SUM(F5:F40)</f>
-        <v/>
+        <v>171252042.23167497</v>
       </c>
     </row>
     <row r="42">
@@ -7325,7 +7325,7 @@
       <c r="E42" s="34" t="n"/>
       <c r="F42" s="36">
         <f>F41*0.08</f>
-        <v/>
+        <v>13700163.378533999</v>
       </c>
     </row>
     <row r="43">
@@ -7340,7 +7340,7 @@
       <c r="E43" s="34" t="n"/>
       <c r="F43" s="36">
         <f>F41*0.03</f>
-        <v/>
+        <v>5137561.266950249</v>
       </c>
     </row>
     <row r="44">
@@ -7355,7 +7355,7 @@
       <c r="E44" s="34" t="n"/>
       <c r="F44" s="36">
         <f>F41*0.05</f>
-        <v/>
+        <v>8562602.111583749</v>
       </c>
     </row>
     <row r="45">
@@ -7370,7 +7370,7 @@
       <c r="E45" s="34" t="n"/>
       <c r="F45" s="36">
         <f>F44*0.19</f>
-        <v/>
+        <v>1626894.4012009122</v>
       </c>
     </row>
     <row r="46">
@@ -7385,7 +7385,7 @@
       <c r="E46" s="28" t="n"/>
       <c r="F46" s="37">
         <f>F41+F42+F43+F44+F45</f>
-        <v/>
+        <v>200279263.38994387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>